<commit_message>
fix: read barcode from sheet inventory of excel
</commit_message>
<xml_diff>
--- a/data/inventory.xlsx
+++ b/data/inventory.xlsx
@@ -1,86 +1,49 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Leonardo Peña\Documents\control_inventario_zg\data\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8FF481A4-1CF0-426D-B4AB-599BE670EC20}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="INVENTARIO" sheetId="1" r:id="rId1"/>
+    <sheet name="INVENTARIO" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <definedNames/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="9">
-  <si>
-    <t>PRODUCTOS</t>
-  </si>
-  <si>
-    <t>ENTRADAS</t>
-  </si>
-  <si>
-    <t>SALIDAS</t>
-  </si>
-  <si>
-    <t>CODIGO</t>
-  </si>
-  <si>
-    <t>PRODUCTO</t>
-  </si>
-  <si>
-    <t>STOCK</t>
-  </si>
-  <si>
-    <t>FECHA</t>
-  </si>
-  <si>
-    <t>CANTIDAD</t>
-  </si>
-  <si>
-    <t>CATEGORIA</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="3">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="0"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <b val="1"/>
+      <color theme="0"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <b val="1"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="9">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -93,7 +56,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.39997558519241921"/>
+        <fgColor theme="8" tint="0.3999755851924192"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -105,19 +68,19 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.59999389629810485"/>
+        <fgColor theme="9" tint="0.5999938962981048"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.39997558519241921"/>
+        <fgColor theme="7" tint="0.3999755851924192"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.79998168889431442"/>
+        <fgColor theme="7" tint="0.7999816888943144"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -140,40 +103,101 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+  <cellXfs count="15">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -439,122 +463,161 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:V3"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:V4"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
-    <col min="8" max="8" width="1.7109375" style="8" customWidth="1"/>
-    <col min="16" max="16" width="1.7109375" style="8" customWidth="1"/>
+    <col width="1.7109375" customWidth="1" style="8" min="8" max="8"/>
+    <col width="14" bestFit="1" customWidth="1" style="12" min="10" max="11"/>
+    <col width="11.28515625" bestFit="1" customWidth="1" style="12" min="12" max="12"/>
+    <col width="10.42578125" bestFit="1" customWidth="1" style="12" min="13" max="13"/>
+    <col width="1.7109375" customWidth="1" style="8" min="16" max="16"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A1" s="12" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="10"/>
-      <c r="C1" s="10"/>
-      <c r="D1" s="10"/>
-      <c r="E1" s="10"/>
-      <c r="F1" s="10"/>
-      <c r="G1" s="4"/>
-      <c r="H1" s="6"/>
-      <c r="J1" s="11" t="s">
-        <v>1</v>
-      </c>
-      <c r="K1" s="10"/>
-      <c r="L1" s="10"/>
-      <c r="M1" s="10"/>
-      <c r="N1" s="10"/>
-      <c r="O1" s="4"/>
-      <c r="P1" s="6"/>
-      <c r="R1" s="9" t="s">
-        <v>2</v>
-      </c>
-      <c r="S1" s="10"/>
-      <c r="T1" s="10"/>
-      <c r="U1" s="10"/>
-      <c r="V1" s="10"/>
+    <row r="1">
+      <c r="A1" s="14" t="inlineStr">
+        <is>
+          <t>PRODUCTOS</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="n"/>
+      <c r="H1" s="6" t="n"/>
+      <c r="J1" s="13" t="inlineStr">
+        <is>
+          <t>ENTRADAS</t>
+        </is>
+      </c>
+      <c r="O1" s="4" t="n"/>
+      <c r="P1" s="6" t="n"/>
+      <c r="R1" s="11" t="inlineStr">
+        <is>
+          <t>SALIDAS</t>
+        </is>
+      </c>
     </row>
-    <row r="2" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A2" s="10"/>
-      <c r="B2" s="10"/>
-      <c r="C2" s="10"/>
-      <c r="D2" s="10"/>
-      <c r="E2" s="10"/>
-      <c r="F2" s="10"/>
-      <c r="G2" s="4"/>
-      <c r="H2" s="6"/>
-      <c r="J2" s="10"/>
-      <c r="K2" s="10"/>
-      <c r="L2" s="10"/>
-      <c r="M2" s="10"/>
-      <c r="N2" s="10"/>
-      <c r="O2" s="4"/>
-      <c r="P2" s="6"/>
-      <c r="R2" s="10"/>
-      <c r="S2" s="10"/>
-      <c r="T2" s="10"/>
-      <c r="U2" s="10"/>
-      <c r="V2" s="10"/>
+    <row r="2">
+      <c r="G2" s="4" t="n"/>
+      <c r="H2" s="6" t="n"/>
+      <c r="O2" s="4" t="n"/>
+      <c r="P2" s="6" t="n"/>
     </row>
-    <row r="3" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="F3" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G3" s="5"/>
-      <c r="H3" s="7"/>
-      <c r="J3" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="K3" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="L3" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="M3" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="N3" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="O3" s="5"/>
-      <c r="P3" s="7"/>
-      <c r="R3" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="S3" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="T3" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="U3" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="V3" s="2" t="s">
-        <v>7</v>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>CODIGO</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t>PRODUCTO</t>
+        </is>
+      </c>
+      <c r="C3" s="1" t="inlineStr">
+        <is>
+          <t>ENTRADAS</t>
+        </is>
+      </c>
+      <c r="D3" s="1" t="inlineStr">
+        <is>
+          <t>CATEGORIA</t>
+        </is>
+      </c>
+      <c r="E3" s="1" t="inlineStr">
+        <is>
+          <t>SALIDAS</t>
+        </is>
+      </c>
+      <c r="F3" s="1" t="inlineStr">
+        <is>
+          <t>STOCK</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="n"/>
+      <c r="H3" s="7" t="n"/>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>CODIGO</t>
+        </is>
+      </c>
+      <c r="K3" s="3" t="inlineStr">
+        <is>
+          <t>PRODUCTO</t>
+        </is>
+      </c>
+      <c r="L3" s="3" t="inlineStr">
+        <is>
+          <t>CATEGORIA</t>
+        </is>
+      </c>
+      <c r="M3" s="3" t="inlineStr">
+        <is>
+          <t>FECHA</t>
+        </is>
+      </c>
+      <c r="N3" s="3" t="inlineStr">
+        <is>
+          <t>CANTIDAD</t>
+        </is>
+      </c>
+      <c r="O3" s="5" t="n"/>
+      <c r="P3" s="7" t="n"/>
+      <c r="R3" s="2" t="inlineStr">
+        <is>
+          <t>CODIGO</t>
+        </is>
+      </c>
+      <c r="S3" s="2" t="inlineStr">
+        <is>
+          <t>PRODUCTO</t>
+        </is>
+      </c>
+      <c r="T3" s="2" t="inlineStr">
+        <is>
+          <t>CATEGORIA</t>
+        </is>
+      </c>
+      <c r="U3" s="2" t="inlineStr">
+        <is>
+          <t>FECHA</t>
+        </is>
+      </c>
+      <c r="V3" s="2" t="inlineStr">
+        <is>
+          <t>CANTIDAD</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="J4" s="10" t="inlineStr">
+        <is>
+          <t>9786075281698</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Manga Berserk</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Manga</t>
+        </is>
+      </c>
+      <c r="M4" s="9" t="n">
+        <v>45551</v>
+      </c>
+      <c r="N4" t="n">
+        <v>11</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="3">
+    <mergeCell ref="J1:N2"/>
     <mergeCell ref="R1:V2"/>
-    <mergeCell ref="J1:N2"/>
     <mergeCell ref="A1:F2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
feat: add write new product
</commit_message>
<xml_diff>
--- a/data/inventory.xlsx
+++ b/data/inventory.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="28680" yWindow="-75" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="INVENTARIO" sheetId="1" state="visible" r:id="rId1"/>
@@ -16,7 +16,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -40,6 +40,14 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
+      <u val="single"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="9">
     <fill>
@@ -103,7 +111,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -115,11 +123,12 @@
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -468,32 +477,32 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V4"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <dimension ref="A1:V22"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="1.7109375" customWidth="1" style="8" min="8" max="8"/>
-    <col width="14" bestFit="1" customWidth="1" style="12" min="10" max="11"/>
-    <col width="11.28515625" bestFit="1" customWidth="1" style="12" min="12" max="12"/>
-    <col width="10.42578125" bestFit="1" customWidth="1" style="12" min="13" max="13"/>
+    <col width="14" bestFit="1" customWidth="1" style="13" min="10" max="11"/>
+    <col width="11.28515625" bestFit="1" customWidth="1" style="13" min="12" max="12"/>
+    <col width="10.42578125" bestFit="1" customWidth="1" style="13" min="13" max="13"/>
     <col width="1.7109375" customWidth="1" style="8" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="14" t="inlineStr">
+      <c r="A1" s="15" t="inlineStr">
         <is>
           <t>PRODUCTOS</t>
         </is>
       </c>
       <c r="G1" s="4" t="n"/>
       <c r="H1" s="6" t="n"/>
-      <c r="J1" s="13" t="inlineStr">
+      <c r="J1" s="12" t="inlineStr">
         <is>
           <t>ENTRADAS</t>
         </is>
       </c>
       <c r="O1" s="4" t="n"/>
       <c r="P1" s="6" t="n"/>
-      <c r="R1" s="11" t="inlineStr">
+      <c r="R1" s="14" t="inlineStr">
         <is>
           <t>SALIDAS</t>
         </is>
@@ -594,24 +603,128 @@
     <row r="4">
       <c r="J4" s="10" t="inlineStr">
         <is>
-          <t>9786075281698</t>
+          <t>7806130008540</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Manga Berserk</t>
+          <t>t</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>Manga</t>
-        </is>
-      </c>
-      <c r="M4" s="9" t="n">
-        <v>45551</v>
+          <t>t</t>
+        </is>
+      </c>
+      <c r="M4" s="9" t="inlineStr">
+        <is>
+          <t>2024-09-30 23:19:31</t>
+        </is>
       </c>
       <c r="N4" t="n">
-        <v>11</v>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>3337875597395</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>2qw</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>sasa</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>2024-10-01 00:03:27</t>
+        </is>
+      </c>
+      <c r="N5" t="n">
+        <v>9</v>
+      </c>
+      <c r="R5" s="11" t="n"/>
+      <c r="S5" s="11" t="n"/>
+      <c r="T5" s="11" t="n"/>
+      <c r="U5" s="11" t="n"/>
+      <c r="V5" s="11" t="n"/>
+    </row>
+    <row r="6">
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>7804930010947</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>lalla</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>alla</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>2024-10-01 00:03:48</t>
+        </is>
+      </c>
+      <c r="N6" t="n">
+        <v>123</v>
+      </c>
+      <c r="R6" s="11" t="n"/>
+      <c r="S6" s="11" t="n"/>
+      <c r="T6" s="11" t="n"/>
+      <c r="U6" s="11" t="n"/>
+      <c r="V6" s="11" t="n"/>
+    </row>
+    <row r="7"/>
+    <row r="8"/>
+    <row r="9"/>
+    <row r="10"/>
+    <row r="11"/>
+    <row r="12"/>
+    <row r="13"/>
+    <row r="14"/>
+    <row r="15"/>
+    <row r="16"/>
+    <row r="17"/>
+    <row r="18"/>
+    <row r="19"/>
+    <row r="20"/>
+    <row r="21">
+      <c r="J21" s="11" t="n"/>
+    </row>
+    <row r="22">
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>3337875597395</t>
+        </is>
+      </c>
+      <c r="S22" t="inlineStr">
+        <is>
+          <t>2qw</t>
+        </is>
+      </c>
+      <c r="T22" t="inlineStr">
+        <is>
+          <t>sasa</t>
+        </is>
+      </c>
+      <c r="U22" t="inlineStr">
+        <is>
+          <t>2024-10-01 01:09:03</t>
+        </is>
+      </c>
+      <c r="V22" t="n">
+        <v>7</v>
       </c>
     </row>
   </sheetData>
@@ -621,5 +734,6 @@
     <mergeCell ref="A1:F2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" paperSize="9"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix: error when read barcode in remove product
</commit_message>
<xml_diff>
--- a/data/inventory.xlsx
+++ b/data/inventory.xlsx
@@ -478,7 +478,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:V22"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col width="1.7109375" customWidth="1" style="8" min="8" max="8"/>
     <col width="14" bestFit="1" customWidth="1" style="13" min="10" max="11"/>
@@ -647,7 +647,7 @@
         </is>
       </c>
       <c r="N5" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="R5" s="11" t="n"/>
       <c r="S5" s="11" t="n"/>
@@ -720,11 +720,11 @@
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>2024-10-01 01:09:03</t>
+          <t>2024-10-01 21:48:49</t>
         </is>
       </c>
       <c r="V22" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>